<commit_message>
Actualización de como se almacenan los datos de output
</commit_message>
<xml_diff>
--- a/configuraciones/Plantilla_credito_A.xlsx
+++ b/configuraciones/Plantilla_credito_A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programación\trabajo\Facturación Electronica Python\InvoicerPRO-Development\configuraciones\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InvoicePRO\invoice-pro-back-local\configuraciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8F32DF-2D3D-48E7-872C-44C6D80BC4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DABDAC-B6BB-4B91-BA33-CE8F538058AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -156,7 +156,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +270,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -727,6 +732,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -736,21 +762,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -775,29 +792,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1444,30 +1449,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="96"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="80"/>
     </row>
     <row r="2" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="99"/>
-      <c r="B2" s="100"/>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
+      <c r="A2" s="100"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
       <c r="E2" s="69"/>
-      <c r="F2" s="97" t="s">
+      <c r="F2" s="81" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="98"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="82"/>
     </row>
     <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
@@ -1488,15 +1493,15 @@
       <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="83"/>
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
       <c r="E4" s="70"/>
       <c r="F4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1504,43 +1509,43 @@
         <v>2</v>
       </c>
       <c r="B5" s="7"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="82"/>
+      <c r="C5" s="98"/>
+      <c r="D5" s="99"/>
       <c r="E5" s="70"/>
       <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="85"/>
-      <c r="H5" s="85"/>
-      <c r="I5" s="86"/>
+      <c r="G5" s="83"/>
+      <c r="H5" s="83"/>
+      <c r="I5" s="90"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="78"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="82"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="99"/>
       <c r="E6" s="9"/>
       <c r="F6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="86"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="83"/>
+      <c r="I6" s="90"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="11"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="84"/>
+      <c r="C7" s="88"/>
+      <c r="D7" s="89"/>
       <c r="E7" s="12"/>
       <c r="F7" s="61" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="11"/>
-      <c r="H7" s="87"/>
-      <c r="I7" s="88"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="92"/>
     </row>
     <row r="8" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
@@ -1628,10 +1633,10 @@
       <c r="A14" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="91" t="s">
+      <c r="B14" s="95" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="91"/>
+      <c r="C14" s="95"/>
       <c r="D14" s="30" t="s">
         <v>19</v>
       </c>
@@ -1878,10 +1883,10 @@
       <c r="D35" s="32"/>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
-      <c r="G35" s="92" t="s">
+      <c r="G35" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="H35" s="92"/>
+      <c r="H35" s="96"/>
       <c r="I35" s="53">
         <f>SUM(I15:I31)</f>
         <v>0</v>
@@ -1893,11 +1898,11 @@
       <c r="C36" s="32"/>
       <c r="D36" s="32"/>
       <c r="E36" s="32"/>
-      <c r="F36" s="92" t="s">
+      <c r="F36" s="96" t="s">
         <v>27</v>
       </c>
-      <c r="G36" s="92"/>
-      <c r="H36" s="92"/>
+      <c r="G36" s="96"/>
+      <c r="H36" s="96"/>
       <c r="I36" s="55">
         <v>0</v>
       </c>
@@ -1909,10 +1914,10 @@
       <c r="D37" s="40"/>
       <c r="E37" s="40"/>
       <c r="F37" s="40"/>
-      <c r="G37" s="93" t="s">
+      <c r="G37" s="97" t="s">
         <v>28</v>
       </c>
-      <c r="H37" s="93"/>
+      <c r="H37" s="97"/>
       <c r="I37" s="54">
         <f>SUM(I35:I36)</f>
         <v>0</v>
@@ -1930,8 +1935,8 @@
       <c r="G38" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="H38" s="89"/>
-      <c r="I38" s="89"/>
+      <c r="H38" s="93"/>
+      <c r="I38" s="93"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="32"/>
@@ -1939,12 +1944,12 @@
       <c r="C39" s="32"/>
       <c r="D39" s="32"/>
       <c r="E39" s="32"/>
-      <c r="F39" s="80" t="s">
+      <c r="F39" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="80"/>
-      <c r="H39" s="90"/>
-      <c r="I39" s="90"/>
+      <c r="G39" s="87"/>
+      <c r="H39" s="94"/>
+      <c r="I39" s="94"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="32"/>
@@ -2043,11 +2048,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:H4"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="C5:D6"/>
@@ -2061,6 +2061,11 @@
     <mergeCell ref="F36:H36"/>
     <mergeCell ref="G37:H37"/>
     <mergeCell ref="G35:H35"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:H4"/>
   </mergeCells>
   <pageMargins left="0.11284722222222222" right="8.6805555555555559E-3" top="0.26041666666666669" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2085,30 +2090,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="96"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="80"/>
     </row>
     <row r="2" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="99"/>
-      <c r="B2" s="100"/>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
+      <c r="A2" s="100"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
       <c r="E2" s="69"/>
-      <c r="F2" s="97" t="s">
+      <c r="F2" s="81" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="98"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="82"/>
     </row>
     <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
@@ -2129,15 +2134,15 @@
       <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="83"/>
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
       <c r="E4" s="70"/>
       <c r="F4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2145,43 +2150,43 @@
         <v>2</v>
       </c>
       <c r="B5" s="7"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="82"/>
+      <c r="C5" s="98"/>
+      <c r="D5" s="99"/>
       <c r="E5" s="70"/>
       <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="85"/>
-      <c r="H5" s="85"/>
-      <c r="I5" s="86"/>
+      <c r="G5" s="83"/>
+      <c r="H5" s="83"/>
+      <c r="I5" s="90"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="78"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="82"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="99"/>
       <c r="E6" s="9"/>
       <c r="F6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="86"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="83"/>
+      <c r="I6" s="90"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="11"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="84"/>
+      <c r="C7" s="88"/>
+      <c r="D7" s="89"/>
       <c r="E7" s="12"/>
       <c r="F7" s="61" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="11"/>
-      <c r="H7" s="87"/>
-      <c r="I7" s="88"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="92"/>
     </row>
     <row r="8" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
@@ -2269,10 +2274,10 @@
       <c r="A14" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="91" t="s">
+      <c r="B14" s="95" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="91"/>
+      <c r="C14" s="95"/>
       <c r="D14" s="30" t="s">
         <v>19</v>
       </c>
@@ -2519,10 +2524,10 @@
       <c r="D35" s="32"/>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
-      <c r="G35" s="92" t="s">
+      <c r="G35" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="H35" s="92"/>
+      <c r="H35" s="96"/>
       <c r="I35" s="53">
         <f>SUM(I15:I31)</f>
         <v>0</v>
@@ -2534,11 +2539,11 @@
       <c r="C36" s="32"/>
       <c r="D36" s="32"/>
       <c r="E36" s="32"/>
-      <c r="F36" s="92" t="s">
+      <c r="F36" s="96" t="s">
         <v>27</v>
       </c>
-      <c r="G36" s="92"/>
-      <c r="H36" s="92"/>
+      <c r="G36" s="96"/>
+      <c r="H36" s="96"/>
       <c r="I36" s="55">
         <v>0</v>
       </c>
@@ -2550,10 +2555,10 @@
       <c r="D37" s="40"/>
       <c r="E37" s="40"/>
       <c r="F37" s="40"/>
-      <c r="G37" s="93" t="s">
+      <c r="G37" s="97" t="s">
         <v>28</v>
       </c>
-      <c r="H37" s="93"/>
+      <c r="H37" s="97"/>
       <c r="I37" s="54">
         <f>SUM(I35:I36)</f>
         <v>0</v>
@@ -2571,8 +2576,8 @@
       <c r="G38" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="H38" s="89"/>
-      <c r="I38" s="89"/>
+      <c r="H38" s="93"/>
+      <c r="I38" s="93"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="32"/>
@@ -2580,12 +2585,12 @@
       <c r="C39" s="32"/>
       <c r="D39" s="32"/>
       <c r="E39" s="32"/>
-      <c r="F39" s="80" t="s">
+      <c r="F39" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="80"/>
-      <c r="H39" s="90"/>
-      <c r="I39" s="90"/>
+      <c r="G39" s="87"/>
+      <c r="H39" s="94"/>
+      <c r="I39" s="94"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="32"/>
@@ -2684,6 +2689,17 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="H7:I7"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="H39:I39"/>
@@ -2691,17 +2707,6 @@
     <mergeCell ref="F36:H36"/>
     <mergeCell ref="G37:H37"/>
     <mergeCell ref="H38:I38"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:H4"/>
   </mergeCells>
   <pageMargins left="0.11284722222222222" right="8.6805555555555559E-3" top="0.26041666666666669" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2726,30 +2731,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="78" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="96"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="80"/>
     </row>
     <row r="2" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="99"/>
-      <c r="B2" s="100"/>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
+      <c r="A2" s="100"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
       <c r="E2" s="69"/>
-      <c r="F2" s="97" t="s">
+      <c r="F2" s="81" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="98"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="82"/>
     </row>
     <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
@@ -2770,15 +2775,15 @@
       <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="83"/>
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
       <c r="E4" s="70"/>
       <c r="F4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2786,43 +2791,43 @@
         <v>2</v>
       </c>
       <c r="B5" s="7"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="82"/>
+      <c r="C5" s="98"/>
+      <c r="D5" s="99"/>
       <c r="E5" s="70"/>
       <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="85"/>
-      <c r="H5" s="85"/>
-      <c r="I5" s="86"/>
+      <c r="G5" s="83"/>
+      <c r="H5" s="83"/>
+      <c r="I5" s="90"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="78"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="82"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="99"/>
       <c r="E6" s="9"/>
       <c r="F6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="86"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="83"/>
+      <c r="I6" s="90"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="11"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="84"/>
+      <c r="C7" s="88"/>
+      <c r="D7" s="89"/>
       <c r="E7" s="12"/>
       <c r="F7" s="61" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="11"/>
-      <c r="H7" s="87"/>
-      <c r="I7" s="88"/>
+      <c r="H7" s="91"/>
+      <c r="I7" s="92"/>
     </row>
     <row r="8" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
@@ -2910,10 +2915,10 @@
       <c r="A14" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="91" t="s">
+      <c r="B14" s="95" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="91"/>
+      <c r="C14" s="95"/>
       <c r="D14" s="30" t="s">
         <v>19</v>
       </c>
@@ -3160,10 +3165,10 @@
       <c r="D35" s="32"/>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
-      <c r="G35" s="92" t="s">
+      <c r="G35" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="H35" s="92"/>
+      <c r="H35" s="96"/>
       <c r="I35" s="53">
         <f>SUM(I15:I31)</f>
         <v>0</v>
@@ -3175,11 +3180,11 @@
       <c r="C36" s="32"/>
       <c r="D36" s="32"/>
       <c r="E36" s="32"/>
-      <c r="F36" s="92" t="s">
+      <c r="F36" s="96" t="s">
         <v>27</v>
       </c>
-      <c r="G36" s="92"/>
-      <c r="H36" s="92"/>
+      <c r="G36" s="96"/>
+      <c r="H36" s="96"/>
       <c r="I36" s="55">
         <v>0</v>
       </c>
@@ -3191,10 +3196,10 @@
       <c r="D37" s="40"/>
       <c r="E37" s="40"/>
       <c r="F37" s="40"/>
-      <c r="G37" s="93" t="s">
+      <c r="G37" s="97" t="s">
         <v>28</v>
       </c>
-      <c r="H37" s="93"/>
+      <c r="H37" s="97"/>
       <c r="I37" s="54">
         <f>SUM(I35:I36)</f>
         <v>0</v>
@@ -3212,8 +3217,8 @@
       <c r="G38" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="H38" s="89"/>
-      <c r="I38" s="89"/>
+      <c r="H38" s="93"/>
+      <c r="I38" s="93"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="32"/>
@@ -3221,12 +3226,12 @@
       <c r="C39" s="32"/>
       <c r="D39" s="32"/>
       <c r="E39" s="32"/>
-      <c r="F39" s="80" t="s">
+      <c r="F39" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="80"/>
-      <c r="H39" s="90"/>
-      <c r="I39" s="90"/>
+      <c r="G39" s="87"/>
+      <c r="H39" s="94"/>
+      <c r="I39" s="94"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="32"/>
@@ -3325,17 +3330,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:H4"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="G5:I5"/>
@@ -3343,6 +3337,17 @@
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="H7:I7"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="H38:I38"/>
   </mergeCells>
   <pageMargins left="0.11284722222222222" right="8.6805555555555559E-3" top="0.26041666666666669" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>